<commit_message>
chore: update note log
update บอกว่าซ่อมไรไปบ้าง
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/Accel_mode.xlsx
+++ b/projects/auto_page/autopageMKII/tables/Accel_mode.xlsx
@@ -497,99 +497,51 @@
       <c r="B14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>26051391VXT8XC</t>
-        </is>
-      </c>
+      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>26051391SJ2W7V</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>26051391J4MAY4</t>
-        </is>
-      </c>
+      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2605139105JNCE</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>260513902AYMY8</t>
-        </is>
-      </c>
+      <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2605138YMAQT9H</t>
-        </is>
-      </c>
+      <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2605138Y7478EW</t>
-        </is>
-      </c>
+      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2605138XC2BH8U</t>
-        </is>
-      </c>
+      <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2605138X21U8WS</t>
-        </is>
-      </c>
+      <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2605138WQSSJPH</t>
-        </is>
-      </c>
+      <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2605138UWVV2QJ</t>
-        </is>
-      </c>
+      <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2605138UXJQEBP</t>
-        </is>
-      </c>
+      <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr"/>
     </row>
     <row r="27">
@@ -601,123 +553,63 @@
       <c r="B27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2605138UPQWH2R</t>
-        </is>
-      </c>
+      <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2605138UBCM0M1</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2605138TYVFTV3</t>
-        </is>
-      </c>
+      <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>2605138TK3B2U5</t>
-        </is>
-      </c>
+      <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>2605138T95RKVP</t>
-        </is>
-      </c>
+      <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>2605138SX22TX3</t>
-        </is>
-      </c>
+      <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2605138SNDGB31</t>
-        </is>
-      </c>
+      <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2605138SAR1QXS</t>
-        </is>
-      </c>
+      <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>2605138S23G5D4</t>
-        </is>
-      </c>
+      <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>2605138RXTJXGH</t>
-        </is>
-      </c>
+      <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>2605128QU09DY9</t>
-        </is>
-      </c>
+      <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>2605128QQAXQP8</t>
-        </is>
-      </c>
+      <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>2605128QQPEYB0</t>
-        </is>
-      </c>
+      <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>2605128QKHV2FB</t>
-        </is>
-      </c>
+      <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>2605128QHXB73Q</t>
-        </is>
-      </c>
+      <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr"/>
     </row>
     <row r="43">
@@ -729,155 +621,79 @@
       <c r="B43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>2605128Q2TVNFK</t>
-        </is>
-      </c>
+      <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>2605128PS147RW</t>
-        </is>
-      </c>
+      <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>2605128PK39BRC</t>
-        </is>
-      </c>
+      <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>2605128PKKFSCQ</t>
-        </is>
-      </c>
+      <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>2605128PA83F79</t>
-        </is>
-      </c>
+      <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>2605128P1V3413</t>
-        </is>
-      </c>
+      <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>2605128NVBPRM4</t>
-        </is>
-      </c>
+      <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>2605128NTDNXHB</t>
-        </is>
-      </c>
+      <c r="A51" t="inlineStr"/>
       <c r="B51" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>2605128NPGRDD5</t>
-        </is>
-      </c>
+      <c r="A52" t="inlineStr"/>
       <c r="B52" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>2605128NCSUN3M</t>
-        </is>
-      </c>
+      <c r="A53" t="inlineStr"/>
       <c r="B53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>2605128MP18464</t>
-        </is>
-      </c>
+      <c r="A54" t="inlineStr"/>
       <c r="B54" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>2605128MN2QME1</t>
-        </is>
-      </c>
+      <c r="A55" t="inlineStr"/>
       <c r="B55" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>2605128MBGJEJV</t>
-        </is>
-      </c>
+      <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>2605128MBR8NDB</t>
-        </is>
-      </c>
+      <c r="A57" t="inlineStr"/>
       <c r="B57" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>2605128M9RBJX0</t>
-        </is>
-      </c>
+      <c r="A58" t="inlineStr"/>
       <c r="B58" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>2605128M5WA495</t>
-        </is>
-      </c>
+      <c r="A59" t="inlineStr"/>
       <c r="B59" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>2605128M32PG5Y</t>
-        </is>
-      </c>
+      <c r="A60" t="inlineStr"/>
       <c r="B60" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>2605128KEXY3M1</t>
-        </is>
-      </c>
+      <c r="A61" t="inlineStr"/>
       <c r="B61" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>2605128KDPVBVT</t>
-        </is>
-      </c>
+      <c r="A62" t="inlineStr"/>
       <c r="B62" t="inlineStr"/>
     </row>
     <row r="63">

</xml_diff>